<commit_message>
Open enrollment: 2,000 points, a drawing, year-round checkup forms, help
- Points total 2,000; confirming a week before the end date adds a
  200-point bonus and a drawing entry
- Checkup forms are welcome all year; the discount starts the month
  after the form is received, so the last-upload deadline is gone
- "Need help?" opens HR booking or sends HR a callback request;
  a "have this ready" list comes before enrolling
- Workbook updated to match, with two new questions to confirm

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REACH_Community_User_Journeys.xlsx
+++ b/REACH_Community_User_Journeys.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>Each step earns points in one open enrollment challenge (up to 825).
+          <t>Each step earns points in one open enrollment challenge (2,000 points in all; confirming a week early adds a drawing entry).
 Tags show HR where each person is, so reminders reach only people still on a step.</t>
         </is>
       </c>
@@ -692,11 +692,11 @@
       <c r="D6" s="24" t="inlineStr">
         <is>
           <t>Complete the sequence, which includes:
-    a. Save the dates (event on the in-app calendar: start, end, last day to upload) +25
-    b. Share what you need: 2-minute needs assessment form. Its User Self-Tagging question adds interest tags, e.g. interest_family, interest_wellness_credit +100
-    c. Reminder to book your personal wellness checkup, with the physician form to download
-    d. Upload a photo of the signed checkup form (Media Upload field) +25; HR approves outside the form and awards +150
-Weekly sequence reminders go to anyone who hasn't finished. Uploads stay open until the last upload day.</t>
+    a. Save the dates (event on the in-app calendar: start and end dates) +50
+    b. Share what you need: 2-minute needs assessment form. Its User Self-Tagging question adds interest tags, e.g. interest_family, interest_wellness_credit +200
+    c. Reminder to turn in your checkup form, or book the visit as soon as you can; forms are welcome all year, and the premium discount starts the month after the form is turned in
+    d. Upload a photo of the signed checkup form (Media Upload field) +100; HR approves outside the form and awards +300
+Weekly sequence reminders go to anyone who hasn't finished.</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
@@ -704,10 +704,10 @@
           <t>Opens 2 weeks before. User sees:
 Your 2027 benefits guide is here. Based on your answers, start with these.
 Displays sequence:
-    a. Explore the new benefits guide: what's new for 2027 (focus content shown by interest tag) +50
-    b. Review your current benefits, then "I've looked" check-in form +50
-    c. Five-minute video on choosing a plan +50
-    d. Same 2 weeks: prompt to the calendar page with dates and sites for one-on-one support at each location; book a virtual time with HR from the calendar (event split into sessions); or join an info session or the fair (QR check-in) +75
+    a. Explore the new benefits guide: what's new for 2027 (focus content shown by interest tag) +150
+    b. Review your current benefits, then "I've looked" check-in form +100
+    c. Five-minute video on choosing a plan +100
+    d. Same 2 weeks: prompt to the calendar page with dates and sites for one-on-one support at each location; book a virtual time with HR from the calendar (event split into sessions); or join an info session or the fair (QR check-in) +150
 Questions go to HR through a short question form.</t>
         </is>
       </c>
@@ -715,9 +715,11 @@
         <is>
           <t>Opens on the enrollment start date. User sees:
 Your 2027 choices are within reach. Enrollment closes [end date].
-    a. Make my choices: Embedded Web Content w/ SSO opens the benefits enrollment site
-    b. "My 2027 choices are made" form; self-tags OE Elections confirmed +200 (+50 in week one)
-    c. You're all set! Thank-you, then a 3-question pulse survey two weeks after close +50
+    a. Have this ready: birth dates and Social Security numbers for anyone you cover, and your doctor's name
+    b. Need help? One tap opens the HR booking calendar; "Call me back" sends the HR admin a push notification with a link to the request and the phone number
+    c. Make my choices: Embedded Web Content w/ SSO opens the benefits enrollment site
+    d. "My 2027 choices are made" form; self-tags OE Elections confirmed +500; +200 and an entry in a random drawing when done at least a week before the end date
+    e. You're all set! Thank-you, then a 3-question pulse survey two weeks after close +150
 HR posts kudos on the news feed when a location reaches 90% confirmed, and checks the confirm form against the enrollment site's completion list each week.
 Interest tags carry into year-round journeys, e.g. "Report a life event" for interest_new_baby.</t>
         </is>
@@ -3815,7 +3817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="20" min="1" max="1"/>
@@ -3928,15 +3930,49 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
+          <t>Call me back</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Adrian's decision: "Call me back" sends the HR admin a push notification with a link to the request and the person's phone number.</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Can a form submission send a push notification to the HR admin, not only an email?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Points and drawing</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Adrian's decision: the challenge is worth 2,000 points, and confirming at least a week before the end date adds an entry in a random drawing.</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>What can 2,000 points buy in the rewards catalog (the cheapest gift card seen was 6,000 points), and who writes and runs the drawing rules?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
           <t>Also to confirm</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>The roster sync needs re-authorizing before the eligibility tags can be relied on, and the phone camera on the upload step wasn't tested.</t>
         </is>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C9" s="28" t="inlineStr">
         <is>
           <t>Who re-authorizes the roster sync, and does the upload step open the phone camera?</t>
         </is>

</xml_diff>

<commit_message>
Open enrollment: the 16-question needs assessment, a message plan, kudos
- The needs assessment is the REACH sixteen-area check-in, linked to
  Know the Need for the full answers
- One enrollment site link shows current benefits and cost, and is
  where people enroll; "you can do this on the clock" in the messages
- 2-week push with a video or flyer and the benefits guide link
- A weekly message plan, two a week at most, reminders stop when done
- Thank each person who confirms; weekly shout-out for locations whose
  whole team is done, in place of the 90% milestone
- Workbook updated to match

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REACH_Community_User_Journeys.xlsx
+++ b/REACH_Community_User_Journeys.xlsx
@@ -685,7 +685,8 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>4 weeks before enrollment opens: scheduled push, text and email "Open enrollment is coming" to everyone tagged OE Eligible (tag comes from the roster sync).
+          <t>4 weeks before enrollment opens: scheduled push, text and email "Get ready for open enrollment" to everyone tagged OE Eligible (tag comes from the roster sync), with the needs survey, the checkup reminder and "Please speak with your manager: you can do this on the clock."
+No more than two messages a week per person, by push or text; each reminder stops once that step is done.
 Post-login focus content takes you straight to the "Needs and checkup" sequence.</t>
         </is>
       </c>
@@ -693,7 +694,7 @@
         <is>
           <t>Complete the sequence, which includes:
     a. Save the dates (event on the in-app calendar: start and end dates) +50
-    b. Share what you need: 2-minute needs assessment form. Its User Self-Tagging question adds interest tags, e.g. interest_family, interest_wellness_credit +200
+    b. Share what you need: the 16-question REACH needs assessment (about 6 minutes, one question per area of life, any can be skipped), so we can plan how to meet personal needs and goals. Each answer is a User Self-Tagging field that adds a tag by area, which points the guide in step 2 to the pages that fit +200
     c. Reminder to turn in your checkup form, or book the visit as soon as you can; forms are welcome all year, and the premium discount starts the month after the form is turned in
     d. Upload a photo of the signed checkup form (Media Upload field) +100; HR approves outside the form and awards +300
 Weekly sequence reminders go to anyone who hasn't finished.</t>
@@ -701,11 +702,10 @@
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>Opens 2 weeks before. User sees:
-Your 2027 benefits guide is here. Based on your answers, start with these.
+          <t>Opens 2 weeks before with a push: "Open enrollment is coming, with some exciting changes", a 60-second video or one-page flyer, and the link to the benefits guide.
 Displays sequence:
     a. Explore the new benefits guide: what's new for 2027 (focus content shown by interest tag) +150
-    b. Review your current benefits, then "I've looked" check-in form +100
+    b. See what you have and pay now: the same enrollment site link used to enroll shows current benefits and cost per paycheck; then "I've looked" check-in form +100
     c. Five-minute video on choosing a plan +100
     d. Same 2 weeks: prompt to the calendar page with dates and sites for one-on-one support at each location; book a virtual time with HR from the calendar (event split into sessions); or join an info session or the fair (QR check-in) +150
 Questions go to HR through a short question form.</t>
@@ -717,10 +717,10 @@
 Your 2027 choices are within reach. Enrollment closes [end date].
     a. Have this ready: birth dates and Social Security numbers for anyone you cover, and your doctor's name
     b. Need help? One tap opens the HR booking calendar; "Call me back" sends the HR admin a push notification with a link to the request and the phone number
-    c. Make my choices: Embedded Web Content w/ SSO opens the benefits enrollment site
+    c. Make my choices: Embedded Web Content w/ SSO opens the same enrollment site that shows what I have and pay now; I can do this on the clock
     d. "My 2027 choices are made" form; self-tags OE Elections confirmed +500; +200 and an entry in a random drawing when done at least a week before the end date
     e. You're all set! Thank-you, then a 3-question pulse survey two weeks after close +150
-HR posts kudos on the news feed when a location reaches 90% confirmed, and checks the confirm form against the enrollment site's completion list each week.
+Each person who confirms gets a thank-you and their points right away; HR posts a weekly shout-out for locations whose whole team is done, and checks the confirm form against the enrollment site's completion list each week.
 Interest tags carry into year-round journeys, e.g. "Report a life event" for interest_new_baby.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Open enrollment: full benefits administration rows and save progress
- Benchmark table gains a "Full benefits administration" group for a
  customer without an enrollment platform or replacing theirs: plans and
  rules, elections, recommendations, pending elections, dependents and
  verification, life events, beneficiaries, evidence of insurability,
  carrier and payroll feeds, ACA, COBRA, plan documents; each sourced
- Save progress: survey and form answers save as you go (build now),
  elections save as pending on the enrollment site; new question to confirm
- Pill key for Next, Later and Skip; workbook updated to match

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REACH_Community_User_Journeys.xlsx
+++ b/REACH_Community_User_Journeys.xlsx
@@ -694,7 +694,7 @@
         <is>
           <t>Complete the sequence, which includes:
     a. Save the dates (event on the in-app calendar: start and end dates) +50
-    b. Share what you need: the 16-question REACH needs assessment (about 6 minutes, one question per area of life, any can be skipped), so we can plan how to meet personal needs and goals. Each answer is a User Self-Tagging field that adds a tag by area, which points the guide in step 2 to the pages that fit +200
+    b. Share what you need: the 16-question REACH needs assessment (about 6 minutes, one question per area of life, any can be skipped, and answers save as you go), so we can plan how to meet personal needs and goals. Each answer is a User Self-Tagging field that adds a tag by area, which points the guide in step 2 to the pages that fit +200
     c. Reminder to turn in your checkup form, or book the visit as soon as you can; forms are welcome all year, and the premium discount starts the month after the form is turned in
     d. Upload a photo of the signed checkup form (Media Upload field) +100; HR approves outside the form and awards +300
 Weekly sequence reminders go to anyone who hasn't finished.</t>
@@ -715,11 +715,12 @@
         <is>
           <t>Opens on the enrollment start date. User sees:
 Your 2027 choices are within reach. Enrollment closes [end date].
-    a. Have this ready: birth dates and Social Security numbers for anyone you cover, and your doctor's name
-    b. Need help? One tap opens the HR booking calendar; "Call me back" sends the HR admin a push notification with a link to the request and the phone number
-    c. Make my choices: Embedded Web Content w/ SSO opens the same enrollment site that shows what I have and pay now; I can do this on the clock
-    d. "My 2027 choices are made" form; self-tags OE Elections confirmed +500; +200 and an entry in a random drawing when done at least a week before the end date
-    e. You're all set! Thank-you, then a 3-question pulse survey two weeks after close +150
+    a. Choices save as pending on the enrollment site until submitted, so the person can stop and come back
+    b. Have this ready: birth dates and Social Security numbers for anyone you cover, and your doctor's name
+    c. Need help? One tap opens the HR booking calendar; "Call me back" sends the HR admin a push notification with a link to the request and the phone number
+    d. Make my choices: Embedded Web Content w/ SSO opens the same enrollment site that shows what I have and pay now; I can do this on the clock
+    e. "My 2027 choices are made" form; self-tags OE Elections confirmed +500; +200 and an entry in a random drawing when done at least a week before the end date
+    f. You're all set! Thank-you, then a 3-question pulse survey two weeks after close +150
 Each person who confirms gets a thank-you and their points right away; HR posts a weekly shout-out for locations whose whole team is done, and checks the confirm form against the enrollment site's completion list each week.
 Interest tags carry into year-round journeys, e.g. "Report a life event" for interest_new_baby.</t>
         </is>
@@ -3817,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="20" min="1" max="1"/>
@@ -3964,15 +3965,32 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
+          <t>Save progress</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>Adrian's decision: progress saves everywhere: finished steps in the journey, each answer in the survey and forms, and choices on the enrollment site.</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>Can a form save answers as the person goes, so a half-finished survey reopens where they stopped? The platform check found no save-and-resume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
           <t>Also to confirm</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>The roster sync needs re-authorizing before the eligibility tags can be relied on, and the phone camera on the upload step wasn't tested.</t>
         </is>
       </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="C10" s="28" t="inlineStr">
         <is>
           <t>Who re-authorizes the roster sync, and does the upload step open the phone camera?</t>
         </is>

</xml_diff>

<commit_message>
Open enrollment: four tags, and no survey section
Sequences already track every step, so the step tags go. Four remain:
OE · Eligible, Need: area, OE · Wellness approved, OE · Confirmed. The
tag chart, tag table, chips and reports follow; reports read sequence
progress and form responses. The needs assessment section is removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REACH_Community_User_Journeys.xlsx
+++ b/REACH_Community_User_Journeys.xlsx
@@ -680,7 +680,7 @@
       <c r="B6" s="25" t="inlineStr">
         <is>
           <t>Each step earns points in one open enrollment challenge (2,000 points in all; confirming a week early adds a drawing entry).
-Tags show HR where each person is, so reminders reach only people still on a step.</t>
+Four tags only: OE Eligible, Need: area, OE Wellness approved, OE Confirmed. Sequences track every step, so steps need no tags.</t>
         </is>
       </c>
       <c r="C6" s="24" t="inlineStr">
@@ -704,7 +704,7 @@
         <is>
           <t>Opens 2 weeks before with a push: "Open enrollment is coming, with some exciting changes", a 60-second video or one-page flyer, and the link to the benefits guide.
 Displays sequence:
-    a. Explore the new benefits guide: what's new for 2027 (focus content shown by interest tag) +150
+    a. Explore the new benefits guide: what's new for 2027 (focus content shown by need tag) +150
     b. See what you have and pay now: the same enrollment site link used to enroll shows current benefits and cost per paycheck; then "I've looked" check-in form +100
     c. Five-minute video on choosing a plan +100
     d. Same 2 weeks: prompt to the calendar page with dates and sites for one-on-one support at each location; book a virtual time with HR from the calendar (event split into sessions); or join an info session or the fair (QR check-in) +150
@@ -719,10 +719,10 @@
     b. Have this ready: birth dates and Social Security numbers for anyone you cover, and your doctor's name
     c. Need help? One tap opens the HR booking calendar; "Call me back" sends the HR admin a push notification with a link to the request and the phone number
     d. Make my choices: Embedded Web Content w/ SSO opens the same enrollment site that shows what I have and pay now; I can do this on the clock
-    e. "My 2027 choices are made" form; self-tags OE Elections confirmed +500; +200 and an entry in a random drawing when done at least a week before the end date
+    e. "My 2027 choices are made" form; self-tags OE Confirmed +500; +200 and an entry in a random drawing when done at least a week before the end date
     f. You're all set! Thank-you, then a 3-question pulse survey two weeks after close +150
 Each person who confirms gets a thank-you and their points right away; HR posts a weekly shout-out for locations whose whole team is done, and checks the confirm form against the enrollment site's completion list each week.
-Interest tags carry into year-round journeys, e.g. "Report a life event" for interest_new_baby.</t>
+Need tags carry into year-round journeys, e.g. "Report a life event" for need_family_care.</t>
         </is>
       </c>
       <c r="G6" s="16" t="n"/>

</xml_diff>

<commit_message>
Open enrollment: fewer sections, sample points, open questions
Removes the tag chart and table and the reports section. Points are
sample values; "what comes after" becomes the journeys we could work
on next; the confirm section is a plain list of open questions, and
the workbook tab is now "Open questions".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REACH_Community_User_Journeys.xlsx
+++ b/REACH_Community_User_Journeys.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions and questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open questions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -749,7 +749,7 @@
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>Assumptions and questions for this example: see the "Assumptions and questions" tab.</t>
+          <t>Open questions for this example: see the "Open questions" tab.</t>
         </is>
       </c>
     </row>
@@ -3818,12 +3818,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="20" min="1" max="1"/>
-    <col width="70" customWidth="1" style="20" min="2" max="2"/>
-    <col width="60" customWidth="1" style="20" min="3" max="3"/>
+    <col width="20" customWidth="1" style="20" min="1" max="1"/>
+    <col width="90" customWidth="1" style="20" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3834,27 +3833,17 @@
       </c>
       <c r="B1" s="26" t="inlineStr">
         <is>
-          <t>Adrian's assumption (platform check, October 21, 2026)</t>
-        </is>
-      </c>
-      <c r="C1" s="26" t="inlineStr">
-        <is>
-          <t>Question to confirm</t>
+          <t>Question</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>Wellness form</t>
+          <t>Checkup form</t>
         </is>
       </c>
       <c r="B2" s="28" t="inlineStr">
-        <is>
-          <t>The platform's upload field takes photos only, and forms have no approval status. The person uploads a photo, and HR approves it outside the form and awards the points by hand.</t>
-        </is>
-      </c>
-      <c r="C2" s="28" t="inlineStr">
         <is>
           <t>Can the upload field take a PDF, can a response carry a pending, approved or sent-back status, and can HR award points by hand?</t>
         </is>
@@ -3863,15 +3852,10 @@
     <row r="3">
       <c r="A3" s="27" t="inlineStr">
         <is>
-          <t>Removing tags</t>
+          <t>Tags</t>
         </is>
       </c>
       <c r="B3" s="28" t="inlineStr">
-        <is>
-          <t>Nothing removes a tag automatically, and a message can't leave out people who have a tag. So the row relies on the sequences' built-in reminders, which go only to people who haven't finished.</t>
-        </is>
-      </c>
-      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>Can a form submission remove a tag, and can an audience leave out people with a tag?</t>
         </is>
@@ -3880,15 +3864,10 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>Reminder timing</t>
+          <t>Reminders</t>
         </is>
       </c>
       <c r="B4" s="28" t="inlineStr">
-        <is>
-          <t>Reminders can only be daily, weekly or monthly, so "every 3 to 4 days" became weekly.</t>
-        </is>
-      </c>
-      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Can a sequence reminder repeat every few days, or is weekly the right rhythm?</t>
         </is>
@@ -3897,15 +3876,10 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>Kudos by location</t>
+          <t>Kudos</t>
         </is>
       </c>
       <c r="B5" s="28" t="inlineStr">
-        <is>
-          <t>The audit found no points totals by location, so HR posts the kudos.</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr">
         <is>
           <t>Is there a report of points or completion by location?</t>
         </is>
@@ -3914,15 +3888,10 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>What it confirmed</t>
+          <t>Enrollment link</t>
         </is>
       </c>
       <c r="B6" s="28" t="inlineStr">
-        <is>
-          <t>Sequences, self-tagging questions, events split into booking slots, and a link type with single sign-on to the enrollment site all exist. Those carry the row.</t>
-        </is>
-      </c>
-      <c r="C6" s="28" t="inlineStr">
         <is>
           <t>How is single sign-on set up for the enrollment link, and does a step hidden by tag drop out of a sequence?</t>
         </is>
@@ -3936,11 +3905,6 @@
       </c>
       <c r="B7" s="28" t="inlineStr">
         <is>
-          <t>Adrian's decision: "Call me back" sends the HR admin a push notification with a link to the request and the person's phone number.</t>
-        </is>
-      </c>
-      <c r="C7" s="28" t="inlineStr">
-        <is>
           <t>Can a form submission send a push notification to the HR admin, not only an email?</t>
         </is>
       </c>
@@ -3948,49 +3912,22 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>Points and drawing</t>
+          <t>Save progress</t>
         </is>
       </c>
       <c r="B8" s="28" t="inlineStr">
         <is>
-          <t>Adrian's decision: the challenge is worth 2,000 points, and confirming at least a week before the end date adds an entry in a random drawing.</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>What can 2,000 points buy in the rewards catalog (the cheapest gift card seen was 6,000 points), and who writes and runs the drawing rules?</t>
+          <t>Can a form save answers as the person goes, so a half-finished survey reopens where they stopped?</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>Save progress</t>
+          <t>Roster and camera</t>
         </is>
       </c>
       <c r="B9" s="28" t="inlineStr">
-        <is>
-          <t>Adrian's decision: progress saves everywhere: finished steps in the journey, each answer in the survey and forms, and choices on the enrollment site.</t>
-        </is>
-      </c>
-      <c r="C9" s="28" t="inlineStr">
-        <is>
-          <t>Can a form save answers as the person goes, so a half-finished survey reopens where they stopped? The platform check found no save-and-resume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t>Also to confirm</t>
-        </is>
-      </c>
-      <c r="B10" s="28" t="inlineStr">
-        <is>
-          <t>The roster sync needs re-authorizing before the eligibility tags can be relied on, and the phone camera on the upload step wasn't tested.</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr">
         <is>
           <t>Who re-authorizes the roster sync, and does the upload step open the phone camera?</t>
         </is>

</xml_diff>

<commit_message>
Open enrollment: benefits administration follows insurance v1 and v2
Team feedback: the In Refresh today cells for full benefits
administration are blank, with a note that some is live in the Refresh
insurance product v1 and most of the rest is in development for v2.
The build-if-replacing plans come out. Adds the universal enrollment
layer and v1/v2 questions, and the next steps (Andy's walkthrough, then
the v2 mapping session). Workbook updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REACH_Community_User_Journeys.xlsx
+++ b/REACH_Community_User_Journeys.xlsx
@@ -3818,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="20" min="1" max="1"/>
@@ -3933,6 +3933,42 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Insurance v1 and v2</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>Which benefits administration features are live in insurance v1, and which are planned for v2?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Universal enrollment layer</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>Could Refresh build one enrollment layer that feeds every major benefits administration platform, and how open and costly are their APIs?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>Andy walks through the Refresh insurance product, then a mapping session for insurance v2 with Andrew Jones, Andy and the team.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Open enrollment: drop the enrollment-layer question and next steps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REACH_Community_User_Journeys.xlsx
+++ b/REACH_Community_User_Journeys.xlsx
@@ -3818,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="20" min="1" max="1"/>
@@ -3945,30 +3945,6 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="27" t="inlineStr">
-        <is>
-          <t>Universal enrollment layer</t>
-        </is>
-      </c>
-      <c r="B11" s="28" t="inlineStr">
-        <is>
-          <t>Could Refresh build one enrollment layer that feeds every major benefits administration platform, and how open and costly are their APIs?</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="27" t="inlineStr">
-        <is>
-          <t>Next</t>
-        </is>
-      </c>
-      <c r="B12" s="28" t="inlineStr">
-        <is>
-          <t>Andy walks through the Refresh insurance product, then a mapping session for insurance v2 with Andrew Jones, Andy and the team.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Open enrollment: how we help 7 in 10 people take part; link-click question
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REACH_Community_User_Journeys.xlsx
+++ b/REACH_Community_User_Journeys.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taking part" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3818,7 +3819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="20" min="1" max="1"/>
@@ -3888,60 +3889,210 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>Enrollment link</t>
+          <t>Link clicks</t>
         </is>
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>How is single sign-on set up for the enrollment link, and does a step hidden by tag drop out of a sequence?</t>
+          <t>Can Refresh count clicks on the enrollment link for each person?</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>Call me back</t>
+          <t>Enrollment link</t>
         </is>
       </c>
       <c r="B7" s="28" t="inlineStr">
         <is>
-          <t>Can a form submission send a push notification to the HR admin, not only an email?</t>
+          <t>How is single sign-on set up for the enrollment link, and does a step hidden by tag drop out of a sequence?</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>Save progress</t>
+          <t>Call me back</t>
         </is>
       </c>
       <c r="B8" s="28" t="inlineStr">
         <is>
-          <t>Can a form save answers as the person goes, so a half-finished survey reopens where they stopped?</t>
+          <t>Can a form submission send a push notification to the HR admin, not only an email?</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>Roster and camera</t>
+          <t>Save progress</t>
         </is>
       </c>
       <c r="B9" s="28" t="inlineStr">
         <is>
-          <t>Who re-authorizes the roster sync, and does the upload step open the phone camera?</t>
+          <t>Can a form save answers as the person goes, so a half-finished survey reopens where they stopped?</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
+          <t>Roster and camera</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>Who re-authorizes the roster sync, and does the upload step open the phone camera?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
           <t>Insurance v1 and v2</t>
         </is>
       </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>Which benefits administration features are live in insurance v1, and which are planned for v2?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="20" min="1" max="1"/>
+    <col width="90" customWidth="1" style="20" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="26" t="inlineStr">
+        <is>
+          <t>How we help</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Goal</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>7 in 10 people take part</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>Count it for each store</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Pick the goal and count it for each store, so we can see which stores need more help.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>Give paid time</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Put the time into each person's schedule, not only in messages; for people paid by the hour, this helps the most.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Make it easy to find</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>A QR code by the time clock and in the break room, and a tablet at team meetings so people can do it on the spot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Celebrate each store</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>The first store where 7 in 10 people take part wins a team prize; thank stores by name in the app's news feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Keep it short</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>About six minutes; any question can be skipped, and answers save as people go.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Use people's own language</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>The survey and messages in Spanish or French where teams need it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>To decide: what counts as taking part</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>It could be finishing the survey, reading the guide, clicking through to the benefits enrollment site, or finishing enrollment. We suggest counting finished surveys and clicks through to the enrollment site: the survey is the part we run, and a click shows someone went to look at their benefits. Refresh can't see whether a person finished enrolling once they're on the site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>To decide: who checks in with each store</t>
+        </is>
+      </c>
       <c r="B10" s="28" t="inlineStr">
         <is>
-          <t>Which benefits administration features are live in insurance v1, and which are planned for v2?</t>
+          <t>The store manager, HR, or a helper chosen at each store.</t>
         </is>
       </c>
     </row>

</xml_diff>